<commit_message>
Verify unchanged 2026 BC election preliminary count on October 28
</commit_message>
<xml_diff>
--- a/client/public/election-data/BC_Election_2026_Riding_Analysis_Preliminary.xlsx
+++ b/client/public/election-data/BC_Election_2026_Riding_Analysis_Preliminary.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive dashboard" sheetId="1" r:id="Rb1759a6322464445"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riding comparison" sheetId="2" r:id="R2a5aa45eff8d42f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional patterns" sheetId="3" r:id="R1d35ce84f15b4559"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NDP seat changes" sheetId="4" r:id="R8b1d1223dbcf470f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closest races" sheetId="5" r:id="Rbf403fbcf4434545"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and sources" sheetId="6" r:id="R41228100a60f4278"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since last snapshot" sheetId="7" r:id="R39b2c0de49e540a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive dashboard" sheetId="1" r:id="R4ad283919c094e15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riding comparison" sheetId="2" r:id="R08ed5d13a8c6400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional patterns" sheetId="3" r:id="R1a6a262c7037460b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NDP seat changes" sheetId="4" r:id="Rf0ec53c396ef4770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closest races" sheetId="5" r:id="R1a400a9f0e9d4360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and sources" sheetId="6" r:id="R912722820bc24ba9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since last snapshot" sheetId="7" r:id="R4cb16492e5784622"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,7 +86,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -123,6 +123,11 @@
         <x:fgColor rgb="FFF4F9F5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4F2F4"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -131,7 +136,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="55">
+  <x:cellXfs count="56">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -215,6 +220,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -236,7 +242,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -479,7 +485,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="18" t="str">
-        <x:v>PRELIMINARY INITIAL COUNT • Elections BC data: 26 Oct 2026, 10:34 (site timestamp) • rechecked 27 Oct: NO NEW DATA • final count planned 6-10 Nov</x:v>
+        <x:v>PRELIMINARY INITIAL COUNT • Elections BC data: 26 Oct 2026, 10:34 (site timestamp) • rechecked 28 Oct: NO NEW DATA • final count planned 6–10 Nov</x:v>
       </x:c>
       <x:c r="B3" s="18"/>
       <x:c r="C3" s="18"/>
@@ -987,7 +993,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="18" t="str">
-        <x:v>Latest official snapshot: 26 Oct 2026, 10:34 (site timestamp) • verified 27 Oct: same data • NDP/Con/Green shares use valid votes</x:v>
+        <x:v>Latest official snapshot: 26 Oct 2026, 10:34 (site timestamp) • verified 28 Oct: same data • NDP/Con/Green shares use valid votes</x:v>
       </x:c>
       <x:c r="B3" s="18"/>
       <x:c r="C3" s="18"/>
@@ -17827,7 +17833,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="18" t="str">
-        <x:v>Public edition | Initial-count data: 26 Oct 2026 | Latest source check: 27 Oct 2026 | Still preliminary</x:v>
+        <x:v>Public edition | Initial-count data: 26 Oct 2026 | Latest source check: 28 Oct 2026 | Still preliminary</x:v>
       </x:c>
       <x:c r="B3" s="18"/>
       <x:c r="C3" s="18"/>
@@ -18018,7 +18024,7 @@
         <x:v>Verification update</x:v>
       </x:c>
       <x:c r="B27" s="40" t="str">
-        <x:v>27 October 2026: official live results page still shows initial-count snapshot dated 26 Oct, 10:34. No new riding-level data or seat-lead changes.</x:v>
+        <x:v>28 October 2026: Elections BC still displays the 26 Oct, 10:34 initial-count snapshot. No new riding-level counts or seat-lead changes since 27 October.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -18034,7 +18040,7 @@
         <x:v>Source status</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>No new official count published as of 27 October check; avoid interpreting unchanged figures as a new vote count.</x:v>
+        <x:v>No new official count published as of the 28 October check; the October 26 source data remains unchanged. This verification is not a new vote count.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18102,7 +18108,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="46" t="str">
-        <x:v>CHECKED 27 OCT 2026  |  LATEST ELECTIONS BC DATA 26 OCT, 10:34  |  NO NEW COUNT PUBLISHED</x:v>
+        <x:v>CHECKED 28 OCT 2026  |  LATEST ELECTIONS BC DATA 26 OCT, 10:34  |  NO NEW COUNT PUBLISHED</x:v>
       </x:c>
       <x:c r="B2" s="46"/>
       <x:c r="C2" s="46"/>
@@ -25782,27 +25788,41 @@
         <x:v>No new release</x:v>
       </x:c>
     </x:row>
-    <x:row r="102" ht="23" customHeight="1">
-      <x:c r="A102" t="str">
+    <x:row r="102" ht="21" customHeight="1">
+      <x:c r="A102" s="55" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c r="B102" s="55" t="str">
+        <x:v>2026-10-26 10:34</x:v>
+      </x:c>
+      <x:c r="C102" s="55" t="n">
+        <x:f>COUNTIF(T6:T98,"UPDATED")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D102" s="55" t="str">
+        <x:v>No new release; unchanged since Oct 27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="22" customHeight="1">
+      <x:c r="A103" t="str">
         <x:v>Final count</x:v>
       </x:c>
-      <x:c r="B102" t="str">
-        <x:v>6-10 Nov 2026</x:v>
-      </x:c>
-      <x:c r="C102"/>
-      <x:c r="D102" t="str">
-        <x:v>Planned, not yet published</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="103" ht="23" customHeight="1">
-      <x:c r="A103" t="str">
-        <x:v>Caveat</x:v>
-      </x:c>
       <x:c r="B103" t="str">
-        <x:v>Any new ballot counts may alter close seats</x:v>
+        <x:v>6–10 Nov 2026</x:v>
       </x:c>
       <x:c r="C103"/>
       <x:c r="D103" t="str">
+        <x:v>Planned, not yet published</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="22" customHeight="1">
+      <x:c r="A104" t="str">
+        <x:v>Caveat</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>Any new ballot counts may alter close seats</x:v>
+      </x:c>
+      <x:c r="D104" t="str">
         <x:v>Not certified</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Refresh October 28 verification of BC election preliminary results
</commit_message>
<xml_diff>
--- a/client/public/election-data/BC_Election_2026_Riding_Analysis_Preliminary.xlsx
+++ b/client/public/election-data/BC_Election_2026_Riding_Analysis_Preliminary.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive dashboard" sheetId="1" r:id="Rb1759a6322464445"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riding comparison" sheetId="2" r:id="R2a5aa45eff8d42f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional patterns" sheetId="3" r:id="R1d35ce84f15b4559"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NDP seat changes" sheetId="4" r:id="R8b1d1223dbcf470f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closest races" sheetId="5" r:id="Rbf403fbcf4434545"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and sources" sheetId="6" r:id="R41228100a60f4278"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since last snapshot" sheetId="7" r:id="R39b2c0de49e540a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive dashboard" sheetId="1" r:id="R4ad283919c094e15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riding comparison" sheetId="2" r:id="R08ed5d13a8c6400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional patterns" sheetId="3" r:id="R1a6a262c7037460b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NDP seat changes" sheetId="4" r:id="Rf0ec53c396ef4770"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closest races" sheetId="5" r:id="R1a400a9f0e9d4360"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and sources" sheetId="6" r:id="R912722820bc24ba9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since last snapshot" sheetId="7" r:id="R4cb16492e5784622"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,7 +86,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -123,6 +123,11 @@
         <x:fgColor rgb="FFF4F9F5"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE4F2F4"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -131,7 +136,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="55">
+  <x:cellXfs count="56">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -215,6 +220,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -236,7 +242,7 @@
         <x:color rgb="FFB91C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -479,7 +485,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="18" t="str">
-        <x:v>PRELIMINARY INITIAL COUNT • Elections BC data: 26 Oct 2026, 10:34 (site timestamp) • rechecked 27 Oct: NO NEW DATA • final count planned 6-10 Nov</x:v>
+        <x:v>PRELIMINARY INITIAL COUNT • Elections BC data: 26 Oct 2026, 10:34 (site timestamp) • rechecked 28 Oct: NO NEW DATA • final count planned 6–10 Nov</x:v>
       </x:c>
       <x:c r="B3" s="18"/>
       <x:c r="C3" s="18"/>
@@ -987,7 +993,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="18" t="str">
-        <x:v>Latest official snapshot: 26 Oct 2026, 10:34 (site timestamp) • verified 27 Oct: same data • NDP/Con/Green shares use valid votes</x:v>
+        <x:v>Latest official snapshot: 26 Oct 2026, 10:34 (site timestamp) • verified 28 Oct: same data • NDP/Con/Green shares use valid votes</x:v>
       </x:c>
       <x:c r="B3" s="18"/>
       <x:c r="C3" s="18"/>
@@ -17827,7 +17833,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="18" t="str">
-        <x:v>Public edition | Initial-count data: 26 Oct 2026 | Latest source check: 27 Oct 2026 | Still preliminary</x:v>
+        <x:v>Public edition | Initial-count data: 26 Oct 2026 | Latest source check: 28 Oct 2026 | Still preliminary</x:v>
       </x:c>
       <x:c r="B3" s="18"/>
       <x:c r="C3" s="18"/>
@@ -18018,7 +18024,7 @@
         <x:v>Verification update</x:v>
       </x:c>
       <x:c r="B27" s="40" t="str">
-        <x:v>27 October 2026: official live results page still shows initial-count snapshot dated 26 Oct, 10:34. No new riding-level data or seat-lead changes.</x:v>
+        <x:v>28 October 2026: Elections BC still displays the 26 Oct, 10:34 initial-count snapshot. No new riding-level counts or seat-lead changes since 27 October.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -18034,7 +18040,7 @@
         <x:v>Source status</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>No new official count published as of 27 October check; avoid interpreting unchanged figures as a new vote count.</x:v>
+        <x:v>No new official count published as of the 28 October check; the October 26 source data remains unchanged. This verification is not a new vote count.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18102,7 +18108,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="46" t="str">
-        <x:v>CHECKED 27 OCT 2026  |  LATEST ELECTIONS BC DATA 26 OCT, 10:34  |  NO NEW COUNT PUBLISHED</x:v>
+        <x:v>CHECKED 28 OCT 2026  |  LATEST ELECTIONS BC DATA 26 OCT, 10:34  |  NO NEW COUNT PUBLISHED</x:v>
       </x:c>
       <x:c r="B2" s="46"/>
       <x:c r="C2" s="46"/>
@@ -25782,27 +25788,41 @@
         <x:v>No new release</x:v>
       </x:c>
     </x:row>
-    <x:row r="102" ht="23" customHeight="1">
-      <x:c r="A102" t="str">
+    <x:row r="102" ht="21" customHeight="1">
+      <x:c r="A102" s="55" t="str">
+        <x:v>2026-10-28</x:v>
+      </x:c>
+      <x:c r="B102" s="55" t="str">
+        <x:v>2026-10-26 10:34</x:v>
+      </x:c>
+      <x:c r="C102" s="55" t="n">
+        <x:f>COUNTIF(T6:T98,"UPDATED")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D102" s="55" t="str">
+        <x:v>No new release; unchanged since Oct 27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="22" customHeight="1">
+      <x:c r="A103" t="str">
         <x:v>Final count</x:v>
       </x:c>
-      <x:c r="B102" t="str">
-        <x:v>6-10 Nov 2026</x:v>
-      </x:c>
-      <x:c r="C102"/>
-      <x:c r="D102" t="str">
-        <x:v>Planned, not yet published</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="103" ht="23" customHeight="1">
-      <x:c r="A103" t="str">
-        <x:v>Caveat</x:v>
-      </x:c>
       <x:c r="B103" t="str">
-        <x:v>Any new ballot counts may alter close seats</x:v>
+        <x:v>6–10 Nov 2026</x:v>
       </x:c>
       <x:c r="C103"/>
       <x:c r="D103" t="str">
+        <x:v>Planned, not yet published</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="22" customHeight="1">
+      <x:c r="A104" t="str">
+        <x:v>Caveat</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>Any new ballot counts may alter close seats</x:v>
+      </x:c>
+      <x:c r="D104" t="str">
         <x:v>Not certified</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Record October 29 election-results verification without new count
</commit_message>
<xml_diff>
--- a/client/public/election-data/BC_Election_2026_Riding_Analysis_Preliminary.xlsx
+++ b/client/public/election-data/BC_Election_2026_Riding_Analysis_Preliminary.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive dashboard" sheetId="1" r:id="R4ad283919c094e15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riding comparison" sheetId="2" r:id="R08ed5d13a8c6400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional patterns" sheetId="3" r:id="R1a6a262c7037460b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NDP seat changes" sheetId="4" r:id="Rf0ec53c396ef4770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closest races" sheetId="5" r:id="R1a400a9f0e9d4360"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and sources" sheetId="6" r:id="R912722820bc24ba9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since last snapshot" sheetId="7" r:id="R4cb16492e5784622"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive dashboard" sheetId="1" r:id="R3620b152acef496d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riding comparison" sheetId="2" r:id="Rd0c5a59387f44a54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional patterns" sheetId="3" r:id="R846a0c7297594625"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NDP seat changes" sheetId="4" r:id="Rbd7cd94a33d44282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closest races" sheetId="5" r:id="Ra3aa25967baa4169"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and sources" sheetId="6" r:id="Rc73a9bc7bcda4e74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since last snapshot" sheetId="7" r:id="Rf673ad7bc84d4621"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="202" formatCode="#,##0;[Red](#,##0);-"/>
     <x:numFmt numFmtId="203" formatCode="#,##0;[Red](#,##0);–"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -85,8 +85,12 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -128,6 +132,11 @@
         <x:fgColor rgb="FFE4F2F4"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFECFDF5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -136,7 +145,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="59">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -221,6 +230,9 @@
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -485,7 +497,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="18" t="str">
-        <x:v>PRELIMINARY INITIAL COUNT • Elections BC data: 26 Oct 2026, 10:34 (site timestamp) • rechecked 28 Oct: NO NEW DATA • final count planned 6–10 Nov</x:v>
+        <x:v>PRELIMINARY INITIAL COUNT • Elections BC data: 26 Oct 2026, 10:34 (site timestamp) • rechecked 29 Oct: NO NEW DATA • final count planned 6–10 Nov</x:v>
       </x:c>
       <x:c r="B3" s="18"/>
       <x:c r="C3" s="18"/>
@@ -17833,7 +17845,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="18" t="str">
-        <x:v>Public edition | Initial-count data: 26 Oct 2026 | Latest source check: 28 Oct 2026 | Still preliminary</x:v>
+        <x:v>Public edition | Initial-count data: 26 Oct 2026 | Latest source check: 29 Oct 2026 | Still preliminary</x:v>
       </x:c>
       <x:c r="B3" s="18"/>
       <x:c r="C3" s="18"/>
@@ -18024,7 +18036,7 @@
         <x:v>Verification update</x:v>
       </x:c>
       <x:c r="B27" s="40" t="str">
-        <x:v>28 October 2026: Elections BC still displays the 26 Oct, 10:34 initial-count snapshot. No new riding-level counts or seat-lead changes since 27 October.</x:v>
+        <x:v>29 October 2026: Elections BC still displays the 26 Oct, 10:34 initial-count snapshot. No new riding-level counts or seat-lead changes since 28 October.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -18040,7 +18052,7 @@
         <x:v>Source status</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>No new official count published as of the 28 October check; the October 26 source data remains unchanged. This verification is not a new vote count.</x:v>
+        <x:v>No new official count published as of the 29 October check; the October 26 source data remains unchanged. This verification is not a new vote count.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18056,10 +18068,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="33" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
@@ -18108,7 +18120,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="46" t="str">
-        <x:v>CHECKED 28 OCT 2026  |  LATEST ELECTIONS BC DATA 26 OCT, 10:34  |  NO NEW COUNT PUBLISHED</x:v>
+        <x:v>CHECKED 29 OCT 2026  |  LATEST ELECTIONS BC DATA 26 OCT, 10:34  |  NO NEW COUNT PUBLISHED</x:v>
       </x:c>
       <x:c r="B2" s="46"/>
       <x:c r="C2" s="46"/>
@@ -25803,26 +25815,42 @@
         <x:v>No new release; unchanged since Oct 27</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" ht="22" customHeight="1">
-      <x:c r="A103" t="str">
+    <x:row r="103" ht="23" customHeight="1">
+      <x:c r="A103" s="57" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="B103" s="57" t="str">
+        <x:v>2026-10-26 10:34</x:v>
+      </x:c>
+      <x:c r="C103" s="57" t="n">
+        <x:f>COUNTIF(T6:T98,"UPDATED")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D103" s="57" t="str">
+        <x:v>No new release; unchanged since Oct 28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="22" customHeight="1">
+      <x:c r="A104" s="58" t="str">
         <x:v>Final count</x:v>
       </x:c>
-      <x:c r="B103" t="str">
+      <x:c r="B104" s="58" t="str">
         <x:v>6–10 Nov 2026</x:v>
       </x:c>
-      <x:c r="C103"/>
-      <x:c r="D103" t="str">
+      <x:c r="C104" s="58"/>
+      <x:c r="D104" s="58" t="str">
         <x:v>Planned, not yet published</x:v>
       </x:c>
     </x:row>
-    <x:row r="104" ht="22" customHeight="1">
-      <x:c r="A104" t="str">
+    <x:row r="105">
+      <x:c r="A105" s="58" t="str">
         <x:v>Caveat</x:v>
       </x:c>
-      <x:c r="B104" t="str">
+      <x:c r="B105" s="58" t="str">
         <x:v>Any new ballot counts may alter close seats</x:v>
       </x:c>
-      <x:c r="D104" t="str">
+      <x:c r="C105" s="58"/>
+      <x:c r="D105" s="58" t="str">
         <x:v>Not certified</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Verify unchanged preliminary BC election results — Oct 29
</commit_message>
<xml_diff>
--- a/client/public/election-data/BC_Election_2026_Riding_Analysis_Preliminary.xlsx
+++ b/client/public/election-data/BC_Election_2026_Riding_Analysis_Preliminary.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive dashboard" sheetId="1" r:id="R4ad283919c094e15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riding comparison" sheetId="2" r:id="R08ed5d13a8c6400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional patterns" sheetId="3" r:id="R1a6a262c7037460b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NDP seat changes" sheetId="4" r:id="Rf0ec53c396ef4770"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closest races" sheetId="5" r:id="R1a400a9f0e9d4360"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and sources" sheetId="6" r:id="R912722820bc24ba9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since last snapshot" sheetId="7" r:id="R4cb16492e5784622"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive dashboard" sheetId="1" r:id="R3620b152acef496d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Riding comparison" sheetId="2" r:id="Rd0c5a59387f44a54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regional patterns" sheetId="3" r:id="R846a0c7297594625"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NDP seat changes" sheetId="4" r:id="Rbd7cd94a33d44282"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closest races" sheetId="5" r:id="Ra3aa25967baa4169"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method and sources" sheetId="6" r:id="Rc73a9bc7bcda4e74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since last snapshot" sheetId="7" r:id="Rf673ad7bc84d4621"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="202" formatCode="#,##0;[Red](#,##0);-"/>
     <x:numFmt numFmtId="203" formatCode="#,##0;[Red](#,##0);–"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -85,8 +85,12 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -128,6 +132,11 @@
         <x:fgColor rgb="FFE4F2F4"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFECFDF5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -136,7 +145,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="59">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -221,6 +230,9 @@
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -485,7 +497,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="18" t="str">
-        <x:v>PRELIMINARY INITIAL COUNT • Elections BC data: 26 Oct 2026, 10:34 (site timestamp) • rechecked 28 Oct: NO NEW DATA • final count planned 6–10 Nov</x:v>
+        <x:v>PRELIMINARY INITIAL COUNT • Elections BC data: 26 Oct 2026, 10:34 (site timestamp) • rechecked 29 Oct: NO NEW DATA • final count planned 6–10 Nov</x:v>
       </x:c>
       <x:c r="B3" s="18"/>
       <x:c r="C3" s="18"/>
@@ -17833,7 +17845,7 @@
     </x:row>
     <x:row r="3" ht="26" customHeight="1">
       <x:c r="A3" s="18" t="str">
-        <x:v>Public edition | Initial-count data: 26 Oct 2026 | Latest source check: 28 Oct 2026 | Still preliminary</x:v>
+        <x:v>Public edition | Initial-count data: 26 Oct 2026 | Latest source check: 29 Oct 2026 | Still preliminary</x:v>
       </x:c>
       <x:c r="B3" s="18"/>
       <x:c r="C3" s="18"/>
@@ -18024,7 +18036,7 @@
         <x:v>Verification update</x:v>
       </x:c>
       <x:c r="B27" s="40" t="str">
-        <x:v>28 October 2026: Elections BC still displays the 26 Oct, 10:34 initial-count snapshot. No new riding-level counts or seat-lead changes since 27 October.</x:v>
+        <x:v>29 October 2026: Elections BC still displays the 26 Oct, 10:34 initial-count snapshot. No new riding-level counts or seat-lead changes since 28 October.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -18040,7 +18052,7 @@
         <x:v>Source status</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>No new official count published as of the 28 October check; the October 26 source data remains unchanged. This verification is not a new vote count.</x:v>
+        <x:v>No new official count published as of the 29 October check; the October 26 source data remains unchanged. This verification is not a new vote count.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -18056,10 +18068,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="33" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="15" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
@@ -18108,7 +18120,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="46" t="str">
-        <x:v>CHECKED 28 OCT 2026  |  LATEST ELECTIONS BC DATA 26 OCT, 10:34  |  NO NEW COUNT PUBLISHED</x:v>
+        <x:v>CHECKED 29 OCT 2026  |  LATEST ELECTIONS BC DATA 26 OCT, 10:34  |  NO NEW COUNT PUBLISHED</x:v>
       </x:c>
       <x:c r="B2" s="46"/>
       <x:c r="C2" s="46"/>
@@ -25803,26 +25815,42 @@
         <x:v>No new release; unchanged since Oct 27</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" ht="22" customHeight="1">
-      <x:c r="A103" t="str">
+    <x:row r="103" ht="23" customHeight="1">
+      <x:c r="A103" s="57" t="str">
+        <x:v>2026-10-29</x:v>
+      </x:c>
+      <x:c r="B103" s="57" t="str">
+        <x:v>2026-10-26 10:34</x:v>
+      </x:c>
+      <x:c r="C103" s="57" t="n">
+        <x:f>COUNTIF(T6:T98,"UPDATED")</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D103" s="57" t="str">
+        <x:v>No new release; unchanged since Oct 28</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="22" customHeight="1">
+      <x:c r="A104" s="58" t="str">
         <x:v>Final count</x:v>
       </x:c>
-      <x:c r="B103" t="str">
+      <x:c r="B104" s="58" t="str">
         <x:v>6–10 Nov 2026</x:v>
       </x:c>
-      <x:c r="C103"/>
-      <x:c r="D103" t="str">
+      <x:c r="C104" s="58"/>
+      <x:c r="D104" s="58" t="str">
         <x:v>Planned, not yet published</x:v>
       </x:c>
     </x:row>
-    <x:row r="104" ht="22" customHeight="1">
-      <x:c r="A104" t="str">
+    <x:row r="105">
+      <x:c r="A105" s="58" t="str">
         <x:v>Caveat</x:v>
       </x:c>
-      <x:c r="B104" t="str">
+      <x:c r="B105" s="58" t="str">
         <x:v>Any new ballot counts may alter close seats</x:v>
       </x:c>
-      <x:c r="D104" t="str">
+      <x:c r="C105" s="58"/>
+      <x:c r="D105" s="58" t="str">
         <x:v>Not certified</x:v>
       </x:c>
     </x:row>

</xml_diff>